<commit_message>
DM profile with email OTP; candidate details (dob/age, education, mobile)
</commit_message>
<xml_diff>
--- a/docs/templates/candidates-template.xlsx
+++ b/docs/templates/candidates-template.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <t>panchayat_samiti</t>
   </si>
@@ -37,6 +37,18 @@
     <t>reservation_category</t>
   </si>
   <si>
+    <t>dob</t>
+  </si>
+  <si>
+    <t>age</t>
+  </si>
+  <si>
+    <t>education</t>
+  </si>
+  <si>
+    <t>mobile</t>
+  </si>
+  <si>
     <t>EXAMPLE - CHURU PANCHAYAT SAMITI</t>
   </si>
   <si>
@@ -55,6 +67,15 @@
     <t>EXAMPLE - सामान्य महिला</t>
   </si>
   <si>
+    <t>15/05/1980</t>
+  </si>
+  <si>
+    <t>स्नातक</t>
+  </si>
+  <si>
+    <t>9876543210</t>
+  </si>
+  <si>
     <t>EXAMPLE - (leave empty for ZP)</t>
   </si>
   <si>
@@ -68,6 +89,9 @@
   </si>
   <si>
     <t>EXAMPLE - अन्य पिछड़ा वर्ग</t>
+  </si>
+  <si>
+    <t>Secondary</t>
   </si>
 </sst>
 </file>
@@ -448,7 +472,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -458,9 +482,13 @@
     <col min="6" max="6" width="18" customWidth="1"/>
     <col min="7" max="7" width="8" customWidth="1"/>
     <col min="8" max="8" width="28" customWidth="1"/>
+    <col min="9" max="9" width="12" customWidth="1"/>
+    <col min="10" max="10" width="5" customWidth="1"/>
+    <col min="11" max="11" width="11" customWidth="1"/>
+    <col min="12" max="12" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -485,13 +513,25 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="C2">
         <v>1</v>
@@ -500,24 +540,33 @@
         <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F2" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G2" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="H2" t="s">
-        <v>13</v>
+        <v>17</v>
+      </c>
+      <c r="I2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K2" t="s">
+        <v>19</v>
+      </c>
+      <c r="L2" t="s">
+        <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="C3">
         <v>1</v>
@@ -526,13 +575,19 @@
         <v>1</v>
       </c>
       <c r="E3" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="G3" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="H3" t="s">
-        <v>18</v>
+        <v>25</v>
+      </c>
+      <c r="J3">
+        <v>45</v>
+      </c>
+      <c r="K3" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ST Format ZP + PS downloads, candidate category, compact warning panel
</commit_message>
<xml_diff>
--- a/docs/templates/candidates-template.xlsx
+++ b/docs/templates/candidates-template.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t>panchayat_samiti</t>
   </si>
@@ -49,6 +49,9 @@
     <t>mobile</t>
   </si>
   <si>
+    <t>candidate_category</t>
+  </si>
+  <si>
     <t>EXAMPLE - CHURU PANCHAYAT SAMITI</t>
   </si>
   <si>
@@ -76,6 +79,9 @@
     <t>9876543210</t>
   </si>
   <si>
+    <t>सामान्य</t>
+  </si>
+  <si>
     <t>EXAMPLE - (leave empty for ZP)</t>
   </si>
   <si>
@@ -92,6 +98,9 @@
   </si>
   <si>
     <t>Secondary</t>
+  </si>
+  <si>
+    <t>OBC</t>
   </si>
 </sst>
 </file>
@@ -472,7 +481,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -486,9 +495,10 @@
     <col min="10" max="10" width="5" customWidth="1"/>
     <col min="11" max="11" width="11" customWidth="1"/>
     <col min="12" max="12" width="12" customWidth="1"/>
+    <col min="13" max="13" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -525,13 +535,16 @@
       <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C2">
         <v>1</v>
@@ -540,33 +553,36 @@
         <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L2" t="s">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="M2" t="s">
+        <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B3" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C3">
         <v>1</v>
@@ -575,19 +591,22 @@
         <v>1</v>
       </c>
       <c r="E3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="H3" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="J3">
         <v>45</v>
       </c>
       <c r="K3" t="s">
-        <v>26</v>
+        <v>28</v>
+      </c>
+      <c r="M3" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Super Admin panel, PS forms, login redesign, TV screen navigation, last booth popup
</commit_message>
<xml_diff>
--- a/docs/templates/candidates-template.xlsx
+++ b/docs/templates/candidates-template.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="49">
   <si>
     <t>panchayat_samiti</t>
   </si>
@@ -52,6 +52,57 @@
     <t>candidate_category</t>
   </si>
   <si>
+    <t>address</t>
+  </si>
+  <si>
+    <t>occupation</t>
+  </si>
+  <si>
+    <t>EXAMPLE note (यह row हटाएँ): Panchayat Samiti का English name (ZP के लिए खाली)</t>
+  </si>
+  <si>
+    <t>PS या ZP</t>
+  </si>
+  <si>
+    <t>Ward no.</t>
+  </si>
+  <si>
+    <t>Ballot position 1, 2, 3…</t>
+  </si>
+  <si>
+    <t>उम्मीदवार का नाम (Hindi)</t>
+  </si>
+  <si>
+    <t>Party short name; निर्दलीय = खाली</t>
+  </si>
+  <si>
+    <t>M / F / O</t>
+  </si>
+  <si>
+    <t>Ward reservation (optional)</t>
+  </si>
+  <si>
+    <t>DOB DD/MM/YYYY (optional)</t>
+  </si>
+  <si>
+    <t>Age, अगर DOB नहीं (optional)</t>
+  </si>
+  <si>
+    <t>Education (optional)</t>
+  </si>
+  <si>
+    <t>10-digit mobile (optional)</t>
+  </si>
+  <si>
+    <t>GEN / SC / ST / OBC (optional)</t>
+  </si>
+  <si>
+    <t>Address (optional)</t>
+  </si>
+  <si>
+    <t>Occupation (optional)</t>
+  </si>
+  <si>
     <t>EXAMPLE - CHURU PANCHAYAT SAMITI</t>
   </si>
   <si>
@@ -80,6 +131,12 @@
   </si>
   <si>
     <t>सामान्य</t>
+  </si>
+  <si>
+    <t>EXAMPLE - ग्राम पोस्ट- साण्डन, तह.- सुजानगढ़, जिला- चूरू</t>
+  </si>
+  <si>
+    <t>कृषि</t>
   </si>
   <si>
     <t>EXAMPLE - (leave empty for ZP)</t>
@@ -481,24 +538,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:O4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="34" customWidth="1"/>
-    <col min="2" max="2" width="10" customWidth="1"/>
-    <col min="4" max="4" width="17" customWidth="1"/>
+    <col min="1" max="1" width="60" customWidth="1"/>
+    <col min="2" max="3" width="10" customWidth="1"/>
+    <col min="4" max="4" width="26" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="18" customWidth="1"/>
-    <col min="7" max="7" width="8" customWidth="1"/>
-    <col min="8" max="8" width="28" customWidth="1"/>
-    <col min="9" max="9" width="12" customWidth="1"/>
-    <col min="10" max="10" width="5" customWidth="1"/>
-    <col min="11" max="11" width="11" customWidth="1"/>
-    <col min="12" max="12" width="12" customWidth="1"/>
-    <col min="13" max="13" width="20" customWidth="1"/>
+    <col min="6" max="6" width="35" customWidth="1"/>
+    <col min="7" max="7" width="11" customWidth="1"/>
+    <col min="8" max="8" width="29" customWidth="1"/>
+    <col min="9" max="9" width="27" customWidth="1"/>
+    <col min="10" max="10" width="30" customWidth="1"/>
+    <col min="11" max="11" width="22" customWidth="1"/>
+    <col min="12" max="12" width="28" customWidth="1"/>
+    <col min="13" max="13" width="32" customWidth="1"/>
+    <col min="14" max="14" width="58" customWidth="1"/>
+    <col min="15" max="15" width="23" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -538,51 +597,66 @@
       <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
+        <v>16</v>
+      </c>
+      <c r="C2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2" t="s">
+        <v>18</v>
       </c>
       <c r="E2" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="G2" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="H2" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="I2" t="s">
-        <v>19</v>
+        <v>23</v>
+      </c>
+      <c r="J2" t="s">
+        <v>24</v>
       </c>
       <c r="K2" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="L2" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="M2" t="s">
-        <v>22</v>
+        <v>27</v>
+      </c>
+      <c r="N2" t="s">
+        <v>28</v>
+      </c>
+      <c r="O2" t="s">
+        <v>29</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="B3" t="s">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="C3">
         <v>1</v>
@@ -591,22 +665,66 @@
         <v>1</v>
       </c>
       <c r="E3" t="s">
-        <v>25</v>
+        <v>32</v>
+      </c>
+      <c r="F3" t="s">
+        <v>33</v>
       </c>
       <c r="G3" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="H3" t="s">
-        <v>27</v>
-      </c>
-      <c r="J3">
+        <v>35</v>
+      </c>
+      <c r="I3" t="s">
+        <v>36</v>
+      </c>
+      <c r="K3" t="s">
+        <v>37</v>
+      </c>
+      <c r="L3" t="s">
+        <v>38</v>
+      </c>
+      <c r="M3" t="s">
+        <v>39</v>
+      </c>
+      <c r="N3" t="s">
+        <v>40</v>
+      </c>
+      <c r="O3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>42</v>
+      </c>
+      <c r="B4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4" t="s">
+        <v>44</v>
+      </c>
+      <c r="G4" t="s">
         <v>45</v>
       </c>
-      <c r="K3" t="s">
-        <v>28</v>
-      </c>
-      <c r="M3" t="s">
-        <v>29</v>
+      <c r="H4" t="s">
+        <v>46</v>
+      </c>
+      <c r="J4">
+        <v>45</v>
+      </c>
+      <c r="K4" t="s">
+        <v>47</v>
+      </c>
+      <c r="M4" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>